<commit_message>
Anpassungen in der Spalte "var_itemformulierung"
</commit_message>
<xml_diff>
--- a/data/missing_meta/missing_meta.xlsx
+++ b/data/missing_meta/missing_meta.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/marco_schuppisser/Desktop/Repository sabseb (new)/metasabseb/data/missing_meta/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78F05E10-1A20-6549-AE13-36597237F4D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{107E5FF8-2E6D-6442-BDD4-FF94BC7BA2B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="68640" yWindow="-3860" windowWidth="38400" windowHeight="23500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8212" uniqueCount="2662">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8242" uniqueCount="2681">
   <si>
     <t>var_defs_key</t>
   </si>
@@ -8524,6 +8524,63 @@
   </si>
   <si>
     <t>Einzelitem: Unterrichtssprache</t>
+  </si>
+  <si>
+    <t>Afrika</t>
+  </si>
+  <si>
+    <t>Asien</t>
+  </si>
+  <si>
+    <t>Andere Sprachregion der Schweiz</t>
+  </si>
+  <si>
+    <t>Europa</t>
+  </si>
+  <si>
+    <t>Lateinamerika (Mittel- und Südamerika)</t>
+  </si>
+  <si>
+    <t>Nordamerika</t>
+  </si>
+  <si>
+    <t>Ozeanien</t>
+  </si>
+  <si>
+    <t>Andere</t>
+  </si>
+  <si>
+    <t>Austauschorganisation (AFS, YFU etc.)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lehrbetrieb </t>
+  </si>
+  <si>
+    <t>Schule</t>
+  </si>
+  <si>
+    <t>eine Gruppenmobilität</t>
+  </si>
+  <si>
+    <t>Mehr als zwei Einzelmobilitäten</t>
+  </si>
+  <si>
+    <t>Mehr als 2 Gruppenmobilität</t>
+  </si>
+  <si>
+    <t>Einzelmobilität als Praktikum</t>
+  </si>
+  <si>
+    <t>Einzelmobilität durch Besuch der lokalen Schule</t>
+  </si>
+  <si>
+    <t>Einzelmobilität in einer Sprachschule</t>
+  </si>
+  <si>
+    <t>zwei Einzelmobilitäten</t>
+  </si>
+  <si>
+    <t>zwei Gruppenmobilitäten</t>
   </si>
 </sst>
 </file>
@@ -8677,7 +8734,17 @@
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
     <cellStyle name="Standard 2" xfId="2" xr:uid="{BC66F5EB-00B7-4041-B960-07C65FD467B2}"/>
   </cellStyles>
-  <dxfs count="44">
+  <dxfs count="18">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C5700"/>
@@ -8685,6 +8752,26 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -8770,16 +8857,6 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
         <color rgb="FF9C5700"/>
       </font>
       <fill>
@@ -8800,16 +8877,6 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
         <color rgb="FF9C0006"/>
       </font>
       <fill>
@@ -8825,276 +8892,6 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -11468,6 +11265,9 @@
       <c r="E54" t="s">
         <v>2199</v>
       </c>
+      <c r="F54" t="s">
+        <v>2673</v>
+      </c>
       <c r="G54" t="s">
         <v>1402</v>
       </c>
@@ -11497,6 +11297,9 @@
       <c r="E55" t="s">
         <v>2199</v>
       </c>
+      <c r="F55" t="s">
+        <v>2674</v>
+      </c>
       <c r="G55" t="s">
         <v>1402</v>
       </c>
@@ -11526,6 +11329,9 @@
       <c r="E56" t="s">
         <v>2199</v>
       </c>
+      <c r="F56" t="s">
+        <v>2675</v>
+      </c>
       <c r="G56" t="s">
         <v>1402</v>
       </c>
@@ -11555,6 +11361,9 @@
       <c r="E57" t="s">
         <v>2199</v>
       </c>
+      <c r="F57" t="s">
+        <v>2676</v>
+      </c>
       <c r="G57" t="s">
         <v>1402</v>
       </c>
@@ -11584,6 +11393,9 @@
       <c r="E58" t="s">
         <v>2199</v>
       </c>
+      <c r="F58" t="s">
+        <v>2677</v>
+      </c>
       <c r="G58" t="s">
         <v>1402</v>
       </c>
@@ -11613,6 +11425,9 @@
       <c r="E59" t="s">
         <v>2199</v>
       </c>
+      <c r="F59" t="s">
+        <v>2678</v>
+      </c>
       <c r="G59" t="s">
         <v>1402</v>
       </c>
@@ -11642,6 +11457,9 @@
       <c r="E60" t="s">
         <v>2199</v>
       </c>
+      <c r="F60" t="s">
+        <v>2679</v>
+      </c>
       <c r="G60" t="s">
         <v>1402</v>
       </c>
@@ -11670,6 +11488,9 @@
       </c>
       <c r="E61" t="s">
         <v>2199</v>
+      </c>
+      <c r="F61" t="s">
+        <v>2680</v>
       </c>
       <c r="G61" t="s">
         <v>1402</v>
@@ -19967,6 +19788,12 @@
       <c r="D320" t="s">
         <v>2646</v>
       </c>
+      <c r="E320" t="s">
+        <v>543</v>
+      </c>
+      <c r="F320" t="s">
+        <v>2669</v>
+      </c>
       <c r="G320" t="s">
         <v>1402</v>
       </c>
@@ -19993,6 +19820,12 @@
       <c r="D321" t="s">
         <v>2646</v>
       </c>
+      <c r="E321" t="s">
+        <v>543</v>
+      </c>
+      <c r="F321" t="s">
+        <v>2670</v>
+      </c>
       <c r="G321" t="s">
         <v>1402</v>
       </c>
@@ -20019,6 +19852,12 @@
       <c r="D322" t="s">
         <v>2646</v>
       </c>
+      <c r="E322" t="s">
+        <v>543</v>
+      </c>
+      <c r="F322" t="s">
+        <v>2671</v>
+      </c>
       <c r="G322" t="s">
         <v>1402</v>
       </c>
@@ -20044,6 +19883,12 @@
       </c>
       <c r="D323" t="s">
         <v>2646</v>
+      </c>
+      <c r="E323" t="s">
+        <v>543</v>
+      </c>
+      <c r="F323" t="s">
+        <v>2672</v>
       </c>
       <c r="G323" t="s">
         <v>1402</v>
@@ -29584,6 +29429,12 @@
       <c r="D585" t="s">
         <v>2653</v>
       </c>
+      <c r="E585" t="s">
+        <v>2276</v>
+      </c>
+      <c r="F585" t="s">
+        <v>2662</v>
+      </c>
       <c r="G585" t="s">
         <v>1402</v>
       </c>
@@ -29610,6 +29461,12 @@
       <c r="D586" t="s">
         <v>2653</v>
       </c>
+      <c r="E586" t="s">
+        <v>2276</v>
+      </c>
+      <c r="F586" t="s">
+        <v>2663</v>
+      </c>
       <c r="G586" t="s">
         <v>1402</v>
       </c>
@@ -29636,6 +29493,12 @@
       <c r="D587" t="s">
         <v>2653</v>
       </c>
+      <c r="E587" t="s">
+        <v>2276</v>
+      </c>
+      <c r="F587" t="s">
+        <v>2664</v>
+      </c>
       <c r="G587" t="s">
         <v>1402</v>
       </c>
@@ -29662,6 +29525,12 @@
       <c r="D588" t="s">
         <v>2653</v>
       </c>
+      <c r="E588" t="s">
+        <v>2276</v>
+      </c>
+      <c r="F588" t="s">
+        <v>2665</v>
+      </c>
       <c r="G588" t="s">
         <v>1402</v>
       </c>
@@ -29688,6 +29557,12 @@
       <c r="D589" t="s">
         <v>2653</v>
       </c>
+      <c r="E589" t="s">
+        <v>2276</v>
+      </c>
+      <c r="F589" t="s">
+        <v>2666</v>
+      </c>
       <c r="G589" t="s">
         <v>1402</v>
       </c>
@@ -29714,6 +29589,12 @@
       <c r="D590" t="s">
         <v>2653</v>
       </c>
+      <c r="E590" t="s">
+        <v>2276</v>
+      </c>
+      <c r="F590" t="s">
+        <v>2667</v>
+      </c>
       <c r="G590" t="s">
         <v>1402</v>
       </c>
@@ -29740,6 +29621,12 @@
       <c r="D591" t="s">
         <v>2653</v>
       </c>
+      <c r="E591" t="s">
+        <v>2276</v>
+      </c>
+      <c r="F591" t="s">
+        <v>2668</v>
+      </c>
       <c r="G591" t="s">
         <v>1402</v>
       </c>
@@ -35057,180 +34944,76 @@
   </sheetData>
   <autoFilter ref="A1:O930" xr:uid="{00000000-0001-0000-0100-000000000000}"/>
   <phoneticPr fontId="4" type="noConversion"/>
-  <conditionalFormatting sqref="A1:O1 A2:J13 L2:O13 A14:O15 A16:J24 L16:O38 A25:I26 A27:J38 A43:J46 L43:O46 K47:O53 A51:I51 A53:I53 A64:J65 L64:O65 K72:O77 A73:I73 J74 A75:I75 J76 A77:I77 A78:O106 A107:I132 K107:O132 A133:O171 A172:I172 K172:O172 A188:J190 L188:O190 A191:O197 A198:H198 J198:O198 A199:O199 A200:H200 J200:O200 A201:O201 A202:H202 J202:O202 A203:O204 A205:H205 J205:O205 A206:O206 A207:H207 J207:O207 A208:O210 A211:H211 J211:O211 A212:O212 A213:H214 J213:O214 A215:O218 A219:H219 J219:O219 A220:O222 A223:H224 J223:O224 A225:O231 A232:J232 L232:O232 A233:O233 A234:J235 L234:O235 A247:I247 K247:O247 A249:I249 K249:O249 K251:O251 K253:O253 K255:O255 A256:J256 L256:O256 A257:O259 A260:J261 L260:O261 A275:H275 J275:O275 A296:H296 J296 L296:O298 A297:C297 A298:H298 J298 A304:H304 L304:O304 A305:O305 A306:H306 L306:O306 A307:O307 A308:H308 L308:O308 A315:H315 L315:O315 A324:H339 L324:O341 A340:I341 A342:O342 A343:I343 L343:O343 A344:O344 A345:I345 L345:O345 A346:O347 A348:I348 K348:O348 A352:I352 K352:O352 A354:I354 K354:O354 A356:I356 K356:O356 A358:J362 L358:O362 A371:J391 L371:O391 A392:O392 A393:J393 L393:O393 A397:I397 L397:O397 L399:O399 L401:O401 L403:O403 L405:O406 A406:J406 A407:O409 A410:J413 L410:O413 L415:O419 A420:O420 A421:J422 L421:O422 A423:O423 L424:O425 L428:O428 L430:O432 L435:O442 A443:H443 A444:J444 L444:O444 A449:J450 L449:O450 A451:O451 A452:J457 L452:O457 A462:J474 L462:O474 A484:J512 L484:O512 A520:J522 L520:O522 L564:O575 A576:O576 A578:J578 L577:O583 A599:J612 L599:O612 A613:O620 A621:J631 L621:O631 A641:J641 L641:O641 A894:J896 L894:O896 A897:O897 A898:J903 L898:O903 A904:O908 A909:I910 K909:O910 A911:O918 J919 A919:I922 K919:O922 A923:J928 L923:O928 A929:O1048576 A39:O42 A54:O63 A66:O71 A72:J72 A74:H74 A76:H76 A173:O187 E297:J297 A309:O314 A316:O323 A349:O351 A353:O353 A355:O355 A357:O357 A475:O475 A514:O514 A523:O527 A537:C537 E537:O537 A529:O536 A528:C528 E528:O528 A47:I49 A50:H50 A52:H52 A584:O598 A632:O640 A394:O396 A398:O398 A400:O400 A402:O402 A404:O404 A399:I399 A401:I401 A403:I403 A405:I405 A416:J419 A428:J428 A435:J436 A415:H415 J415 A438:J442 A437:H437 J437 A424:J425 A430:J432 A414:O414 A429:O429 A433:O434 J443:O443 A445:H445 J445:O445 A446:O448 A426:O427 A458:O461 A478:O483 A476:H477 J476:O477 A513:H513 J513:O513 A518:O519 A517:H517 J517:O517 A516:O516 A515:H515 J515:O515 A564:J564 A546:H546 J546:O546 A570:J571 A574:J575 A568:H569 J568:J569 A572:H573 J572:J573 A538:O545 A547:O563 A567:J567 A565:H566 J565:J566 A577:H577 J577 A580:J583 A579:H579 J579 A236:O246 A248:O248 A250:O250 A252:O252 A254:O254 A251:I251 A253:I253 A255:I255 A363:O370 A642:O893 K495">
-    <cfRule type="expression" dxfId="3" priority="50">
+  <conditionalFormatting sqref="A297:K297">
+    <cfRule type="expression" dxfId="17" priority="1">
+      <formula>ISNUMBER(SEARCH("Nicht in der Skalendokumentation",$O297))</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="16" priority="2">
+      <formula>ISNUMBER(SEARCH("EMPTY DATA COLUMN",$O297))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A1:O1 A2:J13 L2:O13 A14:O15 A16:J24 L16:O38 A25:I26 A27:J38 A39:O42 A43:J46 L43:O46 A47:I49 K47:O53 A50:H50 A51:I51 A52:H52 A53:I53 A54:O63 A64:J65 L64:O65 A66:O71 A72:J72 K72:O77 A73:I73 A74:H74 J74 A75:I75 A76:H76 J76 A77:I77 A78:O106 A107:I132 K107:O132 A133:O171 A172:I172 K172:O172 A173:O187 A188:J190 L188:O190 A191:O197 A198:H198 J198:O198 A199:O199 A200:H200 J200:O200 A201:O201 A202:H202 J202:O202 A203:O204 A205:H205 J205:O205 A206:O206 A207:H207 J207:O207 A208:O210 A211:H211 J211:O211 A212:O212 A213:H214 J213:O214 A215:O218 A219:H219 J219:O219 A220:O222 A223:H224 J223:O224 A225:O231 A232:J232 L232:O232 A233:O233 A234:J235 L234:O235 A236:O246 A247:I247 K247:O247 A248:O248 A249:I249 K249:O249 A250:O250 A251:I251 K251:O251 A252:O252 A253:I253 K253:O253 A254:O254 A255:I255 K255:O255 A256:J256 L256:O256 A257:O259 A260:J261 L260:O261 A275:H275 J275:O275 A296:H296 J296 L296:O298 A298:H298 J298 A304:H304 L304:O304 A305:O305 A306:H306 L306:O306 A307:O307 A308:H308 L308:O308 A309:O314 A315:H315 L315:O315 A324:H339 L324:O341 A340:I341 A342:O342 A343:I343 L343:O343 A344:O344 A345:I345 L345:O345 A346:O347 A348:I348 K348:O348 A349:O351 A352:I352 K352:O352 A353:O353 A354:I354 K354:O354 A355:O355 A356:I356 K356:O356 A357:O357 A358:J362 L358:O362 A363:O370 A371:J391 L371:O391 A392:O392 A393:J393 L393:O393 A394:O396 A397:I397 L397:O397 A398:O398 A399:I399 L399:O399 A400:O400 A401:I401 L401:O401 A402:O402 A403:I403 L403:O403 A404:O404 A405:I405 L405:O406 A406:J406 A407:O409 A410:J413 L410:O413 A414:O414 A415:H415 J415 L415:O419 A416:J419 A420:O420 A421:J422 L421:O422 A423:O423 A424:J425 L424:O425 A426:O427 A428:J428 L428:O428 A429:O429 A430:J432 L430:O432 A433:O434 A435:J436 L435:O442 A437:H437 J437 A438:J442 A443:H443 J443:O443 A444:J444 L444:O444 A445:H445 J445:O445 A446:O448 A449:J450 L449:O450 A451:O451 A452:J457 L452:O457 A458:O461 A462:J474 L462:O474 A475:O475 A476:H477 J476:O477 A478:O483 A484:J512 L484:O512 K495 A513:H513 J513:O513 A514:O514 A515:H515 J515:O515 A516:O516 A517:H517 J517:O517 A518:O519 A520:J522 L520:O522 A523:O527 A528:C528 E528:O528 A529:O536 A537:C537 E537:O537 A538:O545 A546:H546 J546:O546 A547:O563 A564:J564 L564:O575 A565:H566 J565:J566 A567:J567 A568:H569 J568:J569 A570:J571 A572:H573 J572:J573 A574:J575 A576:O576 A577:H577 J577 L577:O583 A578:J578 A579:H579 J579 A580:J583 A599:J612 L599:O612 A613:O620 A621:J631 L621:O631 A632:O640 A641:J641 L641:O641 A642:O893 A894:J896 L894:O896 A897:O897 A898:J903 L898:O903 A904:O908 A909:I910 K909:O910 A911:O918 J919 A919:I922 K919:O922 A923:J928 L923:O928 A929:O1048576 A316:O323 A584:O598">
+    <cfRule type="expression" dxfId="1" priority="51">
+      <formula>ISNUMBER(SEARCH("EMPTY DATA COLUMN",$O1))</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="0" priority="50">
       <formula>ISNUMBER(SEARCH("Nicht in der Skalendokumentation",$O1))</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="2" priority="51">
-      <formula>ISNUMBER(SEARCH("EMPTY DATA COLUMN",$O1))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A262:O274">
-    <cfRule type="expression" dxfId="43" priority="35">
+    <cfRule type="expression" dxfId="15" priority="36">
+      <formula>ISNUMBER(SEARCH("EMPTY DATA COLUMN",$O262))</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="14" priority="35">
       <formula>ISNUMBER(SEARCH("Nicht in der Skalendokumentation",$O262))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="42" priority="36">
-      <formula>ISNUMBER(SEARCH("EMPTY DATA COLUMN",$O262))</formula>
-    </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A276:O276 A281:O282 A277:C280 E277:O280 A284:O284 A283:C283 E283:O283 A286:O287 A285:C285 E285:O285 A290:O290 A288:C289 E288:O289 A294:O294 A291:C293 E291:O293 A295:C295 E295:O295">
-    <cfRule type="expression" dxfId="41" priority="33">
+  <conditionalFormatting sqref="A276:O295">
+    <cfRule type="expression" dxfId="13" priority="5">
       <formula>ISNUMBER(SEARCH("Nicht in der Skalendokumentation",$O276))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="40" priority="34">
+    <cfRule type="expression" dxfId="12" priority="6">
       <formula>ISNUMBER(SEARCH("EMPTY DATA COLUMN",$O276))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A299:O303">
-    <cfRule type="expression" dxfId="39" priority="29">
+    <cfRule type="expression" dxfId="11" priority="30">
+      <formula>ISNUMBER(SEARCH("EMPTY DATA COLUMN",$O299))</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="10" priority="29">
       <formula>ISNUMBER(SEARCH("Nicht in der Skalendokumentation",$O299))</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="38" priority="30">
-      <formula>ISNUMBER(SEARCH("EMPTY DATA COLUMN",$O299))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J26 J920:J922">
-    <cfRule type="expression" dxfId="37" priority="54">
+    <cfRule type="expression" dxfId="9" priority="55">
+      <formula>ISNUMBER(SEARCH("EMPTY DATA COLUMN",$O25))</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="8" priority="54">
       <formula>ISNUMBER(SEARCH("Nicht in der Skalendokumentation",$O25))</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="36" priority="55">
-      <formula>ISNUMBER(SEARCH("EMPTY DATA COLUMN",$O25))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J909:J910">
-    <cfRule type="expression" dxfId="35" priority="58">
+    <cfRule type="expression" dxfId="7" priority="59">
+      <formula>ISNUMBER(SEARCH("EMPTY DATA COLUMN",$O910))</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="6" priority="58">
       <formula>ISNUMBER(SEARCH("Nicht in der Skalendokumentation",$O910))</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="34" priority="59">
-      <formula>ISNUMBER(SEARCH("EMPTY DATA COLUMN",$O910))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K341">
-    <cfRule type="expression" dxfId="33" priority="43">
+    <cfRule type="expression" dxfId="5" priority="44">
+      <formula>ISNUMBER(SEARCH("EMPTY DATA COLUMN",$O341))</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="4" priority="43">
       <formula>ISNUMBER(SEARCH("Nicht in der Skalendokumentation",$O341))</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="32" priority="44">
-      <formula>ISNUMBER(SEARCH("EMPTY DATA COLUMN",$O341))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K923:K928">
-    <cfRule type="expression" dxfId="31" priority="41">
+    <cfRule type="expression" dxfId="3" priority="41">
       <formula>ISNUMBER(SEARCH("Nicht in der Skalendokumentation",$O922))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="30" priority="42">
+    <cfRule type="expression" dxfId="2" priority="42">
       <formula>ISNUMBER(SEARCH("EMPTY DATA COLUMN",$O922))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D277">
-    <cfRule type="expression" dxfId="29" priority="27">
-      <formula>ISNUMBER(SEARCH("Nicht in der Skalendokumentation",$O277))</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="28" priority="28">
-      <formula>ISNUMBER(SEARCH("EMPTY DATA COLUMN",$O277))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D278">
-    <cfRule type="expression" dxfId="27" priority="25">
-      <formula>ISNUMBER(SEARCH("Nicht in der Skalendokumentation",$O278))</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="26" priority="26">
-      <formula>ISNUMBER(SEARCH("EMPTY DATA COLUMN",$O278))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D279">
-    <cfRule type="expression" dxfId="25" priority="23">
-      <formula>ISNUMBER(SEARCH("Nicht in der Skalendokumentation",$O279))</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="24" priority="24">
-      <formula>ISNUMBER(SEARCH("EMPTY DATA COLUMN",$O279))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D280">
-    <cfRule type="expression" dxfId="23" priority="21">
-      <formula>ISNUMBER(SEARCH("Nicht in der Skalendokumentation",$O280))</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="22" priority="22">
-      <formula>ISNUMBER(SEARCH("EMPTY DATA COLUMN",$O280))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D283">
-    <cfRule type="expression" dxfId="21" priority="19">
-      <formula>ISNUMBER(SEARCH("Nicht in der Skalendokumentation",$O283))</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="20" priority="20">
-      <formula>ISNUMBER(SEARCH("EMPTY DATA COLUMN",$O283))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D285">
-    <cfRule type="expression" dxfId="19" priority="17">
-      <formula>ISNUMBER(SEARCH("Nicht in der Skalendokumentation",$O285))</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="18" priority="18">
-      <formula>ISNUMBER(SEARCH("EMPTY DATA COLUMN",$O285))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D288">
-    <cfRule type="expression" dxfId="17" priority="15">
-      <formula>ISNUMBER(SEARCH("Nicht in der Skalendokumentation",$O288))</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="16" priority="16">
-      <formula>ISNUMBER(SEARCH("EMPTY DATA COLUMN",$O288))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D289">
-    <cfRule type="expression" dxfId="15" priority="13">
-      <formula>ISNUMBER(SEARCH("Nicht in der Skalendokumentation",$O289))</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="14" priority="14">
-      <formula>ISNUMBER(SEARCH("EMPTY DATA COLUMN",$O289))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D292">
-    <cfRule type="expression" dxfId="13" priority="11">
-      <formula>ISNUMBER(SEARCH("Nicht in der Skalendokumentation",$O292))</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="12" priority="12">
-      <formula>ISNUMBER(SEARCH("EMPTY DATA COLUMN",$O292))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D291">
-    <cfRule type="expression" dxfId="11" priority="9">
-      <formula>ISNUMBER(SEARCH("Nicht in der Skalendokumentation",$O291))</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="10" priority="10">
-      <formula>ISNUMBER(SEARCH("EMPTY DATA COLUMN",$O291))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D293">
-    <cfRule type="expression" dxfId="9" priority="7">
-      <formula>ISNUMBER(SEARCH("Nicht in der Skalendokumentation",$O293))</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="8" priority="8">
-      <formula>ISNUMBER(SEARCH("EMPTY DATA COLUMN",$O293))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D295">
-    <cfRule type="expression" dxfId="7" priority="5">
-      <formula>ISNUMBER(SEARCH("Nicht in der Skalendokumentation",$O295))</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="6" priority="6">
-      <formula>ISNUMBER(SEARCH("EMPTY DATA COLUMN",$O295))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D297">
-    <cfRule type="expression" dxfId="5" priority="3">
-      <formula>ISNUMBER(SEARCH("Nicht in der Skalendokumentation",$O297))</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="4" priority="4">
-      <formula>ISNUMBER(SEARCH("EMPTY DATA COLUMN",$O297))</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="K297">
-    <cfRule type="expression" dxfId="1" priority="1">
-      <formula>ISNUMBER(SEARCH("Nicht in der Skalendokumentation",$O297))</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="0" priority="2">
-      <formula>ISNUMBER(SEARCH("EMPTY DATA COLUMN",$O297))</formula>
     </cfRule>
   </conditionalFormatting>
   <hyperlinks>

</xml_diff>

<commit_message>
Ober-/Unterthema bezgl. "Statistische Angaben aus XLS-Uploads Teilnehmerliste" angepasst
</commit_message>
<xml_diff>
--- a/data/missing_meta/missing_meta.xlsx
+++ b/data/missing_meta/missing_meta.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/marco_schuppisser/Desktop/Repository sabseb (new)/metasabseb/data/missing_meta/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{107E5FF8-2E6D-6442-BDD4-FF94BC7BA2B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8DD88BCB-E5A9-F24B-8B22-8BAAF39F427E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="68640" yWindow="-3860" windowWidth="38400" windowHeight="23500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8242" uniqueCount="2681">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8248" uniqueCount="2681">
   <si>
     <t>var_defs_key</t>
   </si>
@@ -8737,41 +8737,11 @@
   <dxfs count="18">
     <dxf>
       <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
         <color rgb="FF9C5700"/>
       </font>
       <fill>
         <patternFill>
           <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -8857,6 +8827,16 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF9C5700"/>
       </font>
       <fill>
@@ -8877,6 +8857,16 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF9C0006"/>
       </font>
       <fill>
@@ -8892,6 +8882,16 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -11554,6 +11554,9 @@
         <v>1407</v>
       </c>
       <c r="G63" t="s">
+        <v>1402</v>
+      </c>
+      <c r="H63" t="s">
         <v>2207</v>
       </c>
       <c r="I63" t="s">
@@ -11647,6 +11650,9 @@
         <v>1426</v>
       </c>
       <c r="G66" t="s">
+        <v>1402</v>
+      </c>
+      <c r="H66" t="s">
         <v>2207</v>
       </c>
       <c r="I66" t="s">
@@ -12801,6 +12807,9 @@
         <v>1407</v>
       </c>
       <c r="G106" t="s">
+        <v>1402</v>
+      </c>
+      <c r="H106" t="s">
         <v>2207</v>
       </c>
       <c r="I106" t="s">
@@ -12830,6 +12839,9 @@
         <v>1723</v>
       </c>
       <c r="G107" t="s">
+        <v>1402</v>
+      </c>
+      <c r="H107" t="s">
         <v>2207</v>
       </c>
       <c r="I107" t="s">
@@ -30814,6 +30826,9 @@
         <v>2285</v>
       </c>
       <c r="G638" t="s">
+        <v>1402</v>
+      </c>
+      <c r="H638" t="s">
         <v>2207</v>
       </c>
       <c r="I638" t="s">
@@ -30843,6 +30858,9 @@
         <v>2286</v>
       </c>
       <c r="G639" t="s">
+        <v>1402</v>
+      </c>
+      <c r="H639" t="s">
         <v>2207</v>
       </c>
       <c r="I639" t="s">
@@ -34952,67 +34970,67 @@
       <formula>ISNUMBER(SEARCH("EMPTY DATA COLUMN",$O297))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A1:O1 A2:J13 L2:O13 A14:O15 A16:J24 L16:O38 A25:I26 A27:J38 A39:O42 A43:J46 L43:O46 A47:I49 K47:O53 A50:H50 A51:I51 A52:H52 A53:I53 A54:O63 A64:J65 L64:O65 A66:O71 A72:J72 K72:O77 A73:I73 A74:H74 J74 A75:I75 A76:H76 J76 A77:I77 A78:O106 A107:I132 K107:O132 A133:O171 A172:I172 K172:O172 A173:O187 A188:J190 L188:O190 A191:O197 A198:H198 J198:O198 A199:O199 A200:H200 J200:O200 A201:O201 A202:H202 J202:O202 A203:O204 A205:H205 J205:O205 A206:O206 A207:H207 J207:O207 A208:O210 A211:H211 J211:O211 A212:O212 A213:H214 J213:O214 A215:O218 A219:H219 J219:O219 A220:O222 A223:H224 J223:O224 A225:O231 A232:J232 L232:O232 A233:O233 A234:J235 L234:O235 A236:O246 A247:I247 K247:O247 A248:O248 A249:I249 K249:O249 A250:O250 A251:I251 K251:O251 A252:O252 A253:I253 K253:O253 A254:O254 A255:I255 K255:O255 A256:J256 L256:O256 A257:O259 A260:J261 L260:O261 A275:H275 J275:O275 A296:H296 J296 L296:O298 A298:H298 J298 A304:H304 L304:O304 A305:O305 A306:H306 L306:O306 A307:O307 A308:H308 L308:O308 A309:O314 A315:H315 L315:O315 A324:H339 L324:O341 A340:I341 A342:O342 A343:I343 L343:O343 A344:O344 A345:I345 L345:O345 A346:O347 A348:I348 K348:O348 A349:O351 A352:I352 K352:O352 A353:O353 A354:I354 K354:O354 A355:O355 A356:I356 K356:O356 A357:O357 A358:J362 L358:O362 A363:O370 A371:J391 L371:O391 A392:O392 A393:J393 L393:O393 A394:O396 A397:I397 L397:O397 A398:O398 A399:I399 L399:O399 A400:O400 A401:I401 L401:O401 A402:O402 A403:I403 L403:O403 A404:O404 A405:I405 L405:O406 A406:J406 A407:O409 A410:J413 L410:O413 A414:O414 A415:H415 J415 L415:O419 A416:J419 A420:O420 A421:J422 L421:O422 A423:O423 A424:J425 L424:O425 A426:O427 A428:J428 L428:O428 A429:O429 A430:J432 L430:O432 A433:O434 A435:J436 L435:O442 A437:H437 J437 A438:J442 A443:H443 J443:O443 A444:J444 L444:O444 A445:H445 J445:O445 A446:O448 A449:J450 L449:O450 A451:O451 A452:J457 L452:O457 A458:O461 A462:J474 L462:O474 A475:O475 A476:H477 J476:O477 A478:O483 A484:J512 L484:O512 K495 A513:H513 J513:O513 A514:O514 A515:H515 J515:O515 A516:O516 A517:H517 J517:O517 A518:O519 A520:J522 L520:O522 A523:O527 A528:C528 E528:O528 A529:O536 A537:C537 E537:O537 A538:O545 A546:H546 J546:O546 A547:O563 A564:J564 L564:O575 A565:H566 J565:J566 A567:J567 A568:H569 J568:J569 A570:J571 A572:H573 J572:J573 A574:J575 A576:O576 A577:H577 J577 L577:O583 A578:J578 A579:H579 J579 A580:J583 A599:J612 L599:O612 A613:O620 A621:J631 L621:O631 A632:O640 A641:J641 L641:O641 A642:O893 A894:J896 L894:O896 A897:O897 A898:J903 L898:O903 A904:O908 A909:I910 K909:O910 A911:O918 J919 A919:I922 K919:O922 A923:J928 L923:O928 A929:O1048576 A316:O323 A584:O598">
-    <cfRule type="expression" dxfId="1" priority="51">
+  <conditionalFormatting sqref="A1:O1 A2:J13 L2:O13 A14:O15 A16:J24 L16:O38 A25:I26 A27:J38 A39:O42 A43:J46 L43:O46 A47:I49 K47:O53 A50:H50 A51:I51 A52:H52 A53:I53 A64:J65 L64:O65 A72:J72 K72:O77 A73:I73 A74:H74 J74 A75:I75 A76:H76 J76 A77:I77 A78:O105 A108:I132 K107:O132 A133:O171 A172:I172 K172:O172 A173:O187 A188:J190 L188:O190 A191:O197 A198:H198 J198:O198 A199:O199 A200:H200 J200:O200 A201:O201 A202:H202 J202:O202 A203:O204 A205:H205 J205:O205 A206:O206 A207:H207 J207:O207 A208:O210 A211:H211 J211:O211 A212:O212 A213:H214 J213:O214 A215:O218 A219:H219 J219:O219 A220:O222 A223:H224 J223:O224 A225:O231 A232:J232 L232:O232 A233:O233 A234:J235 L234:O235 A236:O246 A247:I247 K247:O247 A248:O248 A249:I249 K249:O249 A250:O250 A251:I251 K251:O251 A252:O252 A253:I253 K253:O253 A254:O254 A255:I255 K255:O255 A256:J256 L256:O256 A257:O259 A260:J261 L260:O261 A275:H275 J275:O275 A296:H296 J296 L296:O298 A298:H298 J298 A304:H304 L304:O304 A305:O305 A306:H306 L306:O306 A307:O307 A308:H308 L308:O308 A309:O314 A315:H315 L315:O315 A316:O323 A324:H339 L324:O341 A340:I341 A342:O342 A343:I343 L343:O343 A344:O344 A345:I345 L345:O345 A346:O347 A348:I348 K348:O348 A349:O351 A352:I352 K352:O352 A353:O353 A354:I354 K354:O354 A355:O355 A356:I356 K356:O356 A357:O357 A358:J362 L358:O362 A363:O370 A371:J391 L371:O391 A392:O392 A393:J393 L393:O393 A394:O396 A397:I397 L397:O397 A398:O398 A399:I399 L399:O399 A400:O400 A401:I401 L401:O401 A402:O402 A403:I403 L403:O403 A404:O404 A405:I405 L405:O406 A406:J406 A407:O409 A410:J413 L410:O413 A414:O414 A415:H415 J415 L415:O419 A416:J419 A420:O420 A421:J422 L421:O422 A423:O423 A424:J425 L424:O425 A426:O427 A428:J428 L428:O428 A429:O429 A430:J432 L430:O432 A433:O434 A435:J436 L435:O442 A437:H437 J437 A438:J442 A443:H443 J443:O443 A444:J444 L444:O444 A445:H445 J445:O445 A446:O448 A449:J450 L449:O450 A451:O451 A452:J457 L452:O457 A458:O461 A462:J474 L462:O474 A475:O475 A476:H477 J476:O477 A478:O483 A484:J512 L484:O512 K495 A513:H513 J513:O513 A514:O514 A515:H515 J515:O515 A516:O516 A517:H517 J517:O517 A518:O519 A520:J522 L520:O522 A523:O527 A528:C528 E528:O528 A529:O536 A537:C537 E537:O537 A538:O545 A546:H546 J546:O546 A547:O563 A564:J564 L564:O575 A565:H566 J565:J566 A567:J567 A568:H569 J568:J569 A570:J571 A572:H573 J572:J573 A574:J575 A576:O576 A577:H577 J577 L577:O583 A578:J578 A579:H579 J579 A580:J583 A584:O598 A599:J612 L599:O612 A613:O620 A621:J631 L621:O631 A632:O637 A641:J641 L641:O641 A642:O893 A894:J896 L894:O896 A897:O897 A898:J903 L898:O903 A904:O908 A909:I910 K909:O910 A911:O918 J919 A919:I922 K919:O922 A923:J928 L923:O928 A929:O1048576 A54:O63 A66:O71 I106:O106 A106:G107 I107 A640:O640 A638:G639 I638:O639">
+    <cfRule type="expression" dxfId="15" priority="50">
+      <formula>ISNUMBER(SEARCH("Nicht in der Skalendokumentation",$O1))</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="14" priority="51">
       <formula>ISNUMBER(SEARCH("EMPTY DATA COLUMN",$O1))</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="0" priority="50">
-      <formula>ISNUMBER(SEARCH("Nicht in der Skalendokumentation",$O1))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A262:O274">
-    <cfRule type="expression" dxfId="15" priority="36">
+    <cfRule type="expression" dxfId="13" priority="35">
+      <formula>ISNUMBER(SEARCH("Nicht in der Skalendokumentation",$O262))</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="12" priority="36">
       <formula>ISNUMBER(SEARCH("EMPTY DATA COLUMN",$O262))</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="14" priority="35">
-      <formula>ISNUMBER(SEARCH("Nicht in der Skalendokumentation",$O262))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A276:O295">
-    <cfRule type="expression" dxfId="13" priority="5">
+    <cfRule type="expression" dxfId="11" priority="5">
       <formula>ISNUMBER(SEARCH("Nicht in der Skalendokumentation",$O276))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="12" priority="6">
+    <cfRule type="expression" dxfId="10" priority="6">
       <formula>ISNUMBER(SEARCH("EMPTY DATA COLUMN",$O276))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A299:O303">
-    <cfRule type="expression" dxfId="11" priority="30">
+    <cfRule type="expression" dxfId="9" priority="29">
+      <formula>ISNUMBER(SEARCH("Nicht in der Skalendokumentation",$O299))</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="8" priority="30">
       <formula>ISNUMBER(SEARCH("EMPTY DATA COLUMN",$O299))</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="10" priority="29">
-      <formula>ISNUMBER(SEARCH("Nicht in der Skalendokumentation",$O299))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J26 J920:J922">
-    <cfRule type="expression" dxfId="9" priority="55">
+    <cfRule type="expression" dxfId="7" priority="54">
+      <formula>ISNUMBER(SEARCH("Nicht in der Skalendokumentation",$O25))</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="6" priority="55">
       <formula>ISNUMBER(SEARCH("EMPTY DATA COLUMN",$O25))</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="8" priority="54">
-      <formula>ISNUMBER(SEARCH("Nicht in der Skalendokumentation",$O25))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J909:J910">
-    <cfRule type="expression" dxfId="7" priority="59">
+    <cfRule type="expression" dxfId="5" priority="58">
+      <formula>ISNUMBER(SEARCH("Nicht in der Skalendokumentation",$O910))</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="4" priority="59">
       <formula>ISNUMBER(SEARCH("EMPTY DATA COLUMN",$O910))</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="6" priority="58">
-      <formula>ISNUMBER(SEARCH("Nicht in der Skalendokumentation",$O910))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K341">
-    <cfRule type="expression" dxfId="5" priority="44">
+    <cfRule type="expression" dxfId="3" priority="43">
+      <formula>ISNUMBER(SEARCH("Nicht in der Skalendokumentation",$O341))</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="2" priority="44">
       <formula>ISNUMBER(SEARCH("EMPTY DATA COLUMN",$O341))</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="4" priority="43">
-      <formula>ISNUMBER(SEARCH("Nicht in der Skalendokumentation",$O341))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K923:K928">
-    <cfRule type="expression" dxfId="3" priority="41">
+    <cfRule type="expression" dxfId="1" priority="41">
       <formula>ISNUMBER(SEARCH("Nicht in der Skalendokumentation",$O922))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="2" priority="42">
+    <cfRule type="expression" dxfId="0" priority="42">
       <formula>ISNUMBER(SEARCH("EMPTY DATA COLUMN",$O922))</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>